<commit_message>
Auto-fit Mismatches row heights in cheshire workbook
</commit_message>
<xml_diff>
--- a/cheshire_reconciliation_2026-05-04.xlsx
+++ b/cheshire_reconciliation_2026-05-04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://m365x97078969-my.sharepoint.com/personal/sysadmin_wondercorp_jp/Documents/2. Management/Reconciliation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C83988C9-FC5B-4990-BCC1-21AEE0464D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC5115EE-4E02-4041-B9F3-2FDE26B6CD67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="18720" windowHeight="11730" firstSheet="1" activeTab="3" xr2:uid="{EB916A4F-D004-4E5F-9215-97140F81D1CE}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="18720" windowHeight="11730" firstSheet="1" activeTab="3" xr2:uid="{052082AA-2202-42CB-A6E0-A3A2FD2CD4A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Mainframe TRANLIST" sheetId="1" r:id="rId1"/>
@@ -989,7 +989,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ABFBC1B-E972-4F09-8A72-EBEB9C63028A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D611659-01DF-449B-9F74-03DEA319BCBB}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1412,7 +1412,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7B62C2C-F49E-4A6E-B257-52951A5E437C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDCE459-8E4C-46DB-804A-5EBDA7D9BCFB}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1638,7 +1638,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82AC7A1A-4F3F-403C-8E98-0DA2295C561D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD7A172-9EC9-4229-BD46-93B89569AC0F}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1942,7 +1942,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ECA279D-51CC-4213-BC5F-823E07D23F48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7112D77-7680-4E74-A09F-4A50B89D46EB}">
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2004,7 +2004,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="336" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A5" s="18">
         <v>1</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="308" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A6" s="18">
         <v>2</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="266" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="42" x14ac:dyDescent="0.35">
       <c r="A7" s="18">
         <v>3</v>
       </c>

</xml_diff>